<commit_message>
Fresco Marché : « halal » seulement pour les produits qui le sont
Tout le catalogue n'est pas halal. Dans les textes proposés pour les
rayons, « halal » ne reste qu'à côté des produits dont le nom le dit
(kebab de poulet Hünkar, allumettes de poulet, dés de dinde) :

- Charcuterie : « halal » retiré du titre Google et du texte.
- Boucherie, Volaille, Turquie : formulations resserrées sur les
  produits concernés.
- Un contrôle refuse désormais « halal » dans un titre de rayon, ou
  ailleurs qu'à côté d'un produit nommé.

L'onglet « À régler à part » signale les 5 descriptions Google en ligne
qui présentent un rayon entier comme halal, et 15 fiches « Certifié
halal » à vérifier sur l'emballage. La règle est ajoutée au panel SEO.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RPCkUuFHpse6kePaQ9QfPW
</commit_message>
<xml_diff>
--- a/fresco-marche/textes-rayons.xlsx
+++ b/fresco-marche/textes-rayons.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Charcuterie de volaille et de bœuf pour sandwichs, pizzas et plats : délices de poulet et de dinde, bacon et lardons de volaille, chorizo, saucisson, salami, ainsi que les spécialités turques sucuk et pastirma. Isla Délice et d'autres marques, avec de nombreuses références halal. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Charcuterie de volaille et de bœuf pour sandwichs, pizzas et plats : délices de poulet et de dinde, bacon et lardons de volaille, chorizo, saucisson, salami, ainsi que les spécialités turques sucuk et pastirma. Isla Délice, Çesnili, Sibel et d'autres marques. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Charcuterie halal de volaille et bœuf | Fresco Marché</t>
+          <t>Charcuterie de volaille et de bœuf pour pros | Fresco Marché</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -850,12 +850,12 @@
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>« halal » dans le title : à garder seulement si toutes les références du rayon sont halal (certificats fournisseurs).</t>
+          <t>Tout le rayon n'est pas halal : « halal » est retiré du titre et du texte. La description Google actuelle du site dit « Charcuterie halal » pour tout le rayon : à remplacer en priorité.</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="100.5" customHeight="1">
+    <row r="7" ht="141" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -879,7 +879,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Viandes pour la restauration rapide : viande de kebab de poulet et lamelles bœuf-volaille Hünkar (surgelé halal), steaks hachés 100 % pur bœuf et burgers de bœuf Biladi en 800 g, dés et allumettes de poulet ou de dinde halal, délices de volaille en tranches. Détail par espèce dans les rayons Volaille et Bœuf. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Viandes pour la restauration rapide : viande de kebab de poulet Hünkar en 800 g (surgelé halal), lamelles de kebab bœuf-volaille Hünkar, steaks hachés 100 % pur bœuf et burgers de bœuf Biladi en 800 g, allumettes de poulet et dés de dinde halal, délices de volaille en tranches. Détail par espèce dans les rayons Volaille et Bœuf. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -904,12 +904,12 @@
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Aucune viande fraîche n'est en ligne dans ce rayon : si vous en vendez, publiez-la ; sinon, le nom « Boucherie » promet plus que ce qu'on trouve.</t>
+          <t>Aucune viande fraîche n'est en ligne dans ce rayon : si vous en vendez, publiez-la ; sinon, le nom « Boucherie » promet plus que ce qu'on trouve. « Halal » n'est écrit que pour les produits dont le nom le dit (kebab de poulet Hünkar, allumettes de poulet, dés de dinde). La description Google actuelle dit « surgelés halal » pour tout le rayon : elle est remplacée.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="73.5" customHeight="1">
+    <row r="8" ht="87" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -933,7 +933,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Volaille pour snacks et restaurants : viande de kebab de poulet Hünkar en 800 g (surgelé halal), dés et allumettes de poulet ou de dinde halal, délices et tranchés de poulet et de dinde pour les sandwichs. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Volaille pour snacks et restaurants : viande de kebab de poulet Hünkar en 800 g (surgelé halal), allumettes de poulet et dés de dinde halal, délices et tranchés de poulet et de dinde pour les sandwichs. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Kebab de poulet Hünkar surgelé halal, dés et allumettes de poulet, délices de dinde et de poulet… La volaille des snacks et restaurants, commande pro.</t>
+          <t>Kebab de poulet Hünkar surgelé halal, allumettes de poulet, dés de dinde, délices de dinde et de poulet… La volaille des snacks et restaurants, commande pro.</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>La marque s'écrit « Hunkar » sur les fiches kebab et « Hünkar » sur d'autres : choisir une seule orthographe.</t>
+          <t>La marque s'écrit « Hunkar » sur les fiches kebab et « Hünkar » sur d'autres : choisir une seule orthographe. La description Google actuelle dit « Surgelés halal » pour tout le rayon : elle est remplacée.</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr"/>
@@ -1010,7 +1010,11 @@
           <t>Steaks hachés 100 % pur bœuf, burgers Biladi nature ou à l'oignon 800 g, lamelles de kebab Hünkar : le bœuf surgelé des snacks, en commande pro à Clichy.</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>La description Google actuelle dit « surgelés halal » ; aucun de ces produits ne l'indique dans son nom. Elle est remplacée.</t>
+        </is>
+      </c>
       <c r="L9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="87" customHeight="1">
@@ -1295,7 +1299,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Produits turcs pour kebabs, durums et mezzés : concentré de tomate Tamek, galettes durum de 30 cm, viande de kebab Hünkar (surgelé halal), sucuk, pastirma de Kayseri, fromage traditionnel Erzurum et yaourt à la grecque en 1 kg. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Produits turcs pour kebabs, durums et mezzés : concentré de tomate Tamek, galettes durum de 30 cm, viande de kebab de poulet Hünkar (surgelé halal), sucuk, pastirma de Kayseri, fromage traditionnel Erzurum et yaourt à la grecque en 1 kg. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1784,7 +1788,11 @@
           <t>Sucuk en tranches, pastirma de Kayseri, salamis aux épices, saucisses bœuf-poulet Sibel… La charcuterie turque des snacks et restaurants, en commande pro.</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>La description Google actuelle parle de « délices halal » : elle est remplacée, sans mention halal.</t>
+        </is>
+      </c>
       <c r="L24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="87" customHeight="1">
@@ -1931,7 +1939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2047,29 +2055,36 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Aucun prix, aucune ville ni aucun délai de livraison non confirmé n'est cité. « Halal » n'est écrit que pour des produits dont le nom le dit, ou pour la marque Isla Délice (voir colonne K).</t>
+          <t>Aucun prix, aucune ville ni aucun délai de livraison non confirmé n'est cité.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr"/>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Tout le catalogue n'est pas halal : « halal » n'est jamais écrit pour un rayon entier, ni dans un titre Google. Il n'apparaît qu'à côté des produits dont le nom le dit (kebab de poulet Hünkar « surgelé halal », allumettes de poulet halal, dés de dinde halal).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Source des chiffres</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>« Produits en ligne » : produits publiés sur la boutique en ligne et visibles dans le rayon, comptés sur frescomarche.fr le 13/10/2026. Le compteur de l'admin Shopify est souvent plus élevé : il inclut les produits non publiés.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>« Produits en ligne » : produits publiés sur la boutique en ligne et visibles dans le rayon, comptés sur frescomarche.fr le 13/10/2026. Le compteur de l'admin Shopify est souvent plus élevé : il inclut les produits non publiés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>« AVANT » : texte, titre et description relevés sur le site le 13/10/2026.</t>
         </is>
@@ -2086,7 +2101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2117,56 +2132,56 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="46.5" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>« Halal » sur des rayons entiers (en ligne aujourd'hui)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Les descriptions Google actuelles de Charcuterie (« Charcuterie halal en tranches »), Boucherie et Volaille (« surgelés halal »), Bœuf (« surgelés halal ») et Charcuterie turque (« délices halal ») présentent tout le rayon comme halal.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Coller en priorité les nouvelles descriptions Google de ces 5 rayons (onglet Rayons, colonne J) : aucune ne présente le rayon entier comme halal.</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3" ht="87" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>15 fiches « Certifié halal »</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>15 fiches disent « Certifié halal » dans leur description sans que le nom du produit le précise : bacons de dinde, blanc de poulet doré, Deliss' Original, délices de dinde et de poulet, lardons de volaille, salami de dinde, Saveurdélice volaille et bœuf aux olives, Tosun pastirma, tranchettes piquantes, tranché de poulet et dinde.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Vérifier sur chaque emballage la mention et l'organisme de certification. Si ce n'est pas écrit sur l'emballage, retirer « Certifié halal » de la fiche.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4" ht="46.5" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Prix visibles dans les filtres</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Sur les pages rayon, le filtre « Precio » affiche le prix le plus élevé (7,50 € pour les fruits) et permet de filtrer par prix : les tarifs réservés aux pros sont visibles de tous.</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Appli Search &amp; Discovery › Filtres : supprimer le filtre de prix.</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr"/>
-    </row>
-    <row r="3" ht="33" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Filtres en espagnol</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Les filtres s'appellent « Disponibilidad » et « Precio ».</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Search &amp; Discovery › Filtres : renommer en « Disponibilité » (et « Prix » si le filtre est gardé).</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4" ht="33" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Poissonnerie</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>0 produit en ligne. La page est indexable et sa description Google promet « poissons et produits de la mer frais et surgelés ».</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Masquer la collection du canal Boutique en ligne tant qu'elle est vide, ou publier les produits.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr"/>
@@ -2174,17 +2189,17 @@
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Arrivages Rungis</t>
+          <t>Filtres en espagnol</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>0 produit en ligne. Le texte annonce « produits arrivés ce matin directement de Rungis… mise à jour chaque matin à 00h01 ».</t>
+          <t>Les filtres s'appellent « Disponibilidad » et « Precio ».</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Même chose que Poissonnerie. Une fois alimenté, ce rayon vaut la peine d'être travaillé : « Rungis » est un argument fort.</t>
+          <t>Search &amp; Discovery › Filtres : renommer en « Disponibilité » (et « Prix » si le filtre est gardé).</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
@@ -2192,35 +2207,35 @@
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Asie</t>
+          <t>Poissonnerie</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2 produits en ligne (aloe vera, coco à boire). La description Google promet « sauces, condiments et ingrédients » d'Asie.</t>
+          <t>0 produit en ligne. La page est indexable et sa description Google promet « poissons et produits de la mer frais et surgelés ».</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Publier les produits asiatiques, ou masquer le rayon en attendant.</t>
+          <t>Masquer la collection du canal Boutique en ligne tant qu'elle est vide, ou publier les produits.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="46.5" customHeight="1">
+    <row r="7" ht="33" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Note interne sur les autres rayons</t>
+          <t>Arrivages Rungis</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>52 autres rayons, hors de ce tableau, affichent encore « Collection automatique … Parent : … » (ex. Agrumes, Bacon-lardons, Bouillons, Cafés-thés).</t>
+          <t>0 produit en ligne. Le texte annonce « produits arrivés ce matin directement de Rungis… mise à jour chaque matin à 00h01 ».</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Après ces 25 rayons : écrire un texte court pour les sous-rayons utiles, et vider la description des autres.</t>
+          <t>Même chose que Poissonnerie. Une fois alimenté, ce rayon vaut la peine d'être travaillé : « Rungis » est un argument fort.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr"/>
@@ -2228,17 +2243,17 @@
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Produits non publiés</t>
+          <t>Asie</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Beaucoup de produits des rayons ne sont pas publiés en ligne (ex. Boissons : 13 en ligne sur 182 dans l'admin).</t>
+          <t>2 produits en ligne (aloe vera, coco à boire). La description Google promet « sauces, condiments et ingrédients » d'Asie.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Publier les produits prêts : chaque rayon en devient plus utile pour les clients et pour Google.</t>
+          <t>Publier les produits asiatiques, ou masquer le rayon en attendant.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
@@ -2246,20 +2261,56 @@
     <row r="9" ht="46.5" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Note interne sur les autres rayons</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>52 autres rayons, hors de ce tableau, affichent encore « Collection automatique … Parent : … » (ex. Agrumes, Bacon-lardons, Bouillons, Cafés-thés).</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Après ces 25 rayons : écrire un texte court pour les sous-rayons utiles, et vider la description des autres.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="33" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Produits non publiés</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Beaucoup de produits des rayons ne sont pas publiés en ligne (ex. Boissons : 13 en ligne sur 182 dans l'admin).</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Publier les produits prêts : chaque rayon en devient plus utile pour les clients et pour Google.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="46.5" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Nom de produit à corriger</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>« Cerneaux de noix extra invalide 250g Profruit » (le mot « invalide » vient sans doute de l'import) ; « COUCOUS MOYEN DARI 1KG » (faute et majuscules).</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Renommer : « Cerneaux de noix extra 250 g Profruit », « Couscous moyen Dari 1 kg ».</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fresco Marché : tout le catalogue est halal
Rachid confirme que tout le catalogue est halal (sa réponse précédente
disait le contraire). « Halal » revient là où les clients le cherchent :

- Titres et descriptions Google : Charcuterie, Boucherie (« Viande
  halal »), Volaille, Bœuf, Charcuterie turque.
- Textes : ces rayons et Surgelés (viandes halal).
- Rien n'est ajouté là où le mot n'apporte rien (fruits, boissons,
  hygiène) ; le contrôle automatique le vérifie.

L'onglet « À régler à part » ne garde qu'un point halal : aucun
organisme de certification n'est cité sur le site. Le panel SEO est mis
à jour (catalogue entièrement halal, à mettre en avant).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RPCkUuFHpse6kePaQ9QfPW
</commit_message>
<xml_diff>
--- a/fresco-marche/textes-rayons.xlsx
+++ b/fresco-marche/textes-rayons.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Charcuterie de volaille et de bœuf pour sandwichs, pizzas et plats : délices de poulet et de dinde, bacon et lardons de volaille, chorizo, saucisson, salami, ainsi que les spécialités turques sucuk et pastirma. Isla Délice, Çesnili, Sibel et d'autres marques. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Charcuterie halal de volaille et de bœuf pour sandwichs, pizzas et plats : délices de poulet et de dinde, bacon et lardons de volaille, chorizo, saucisson, salami, ainsi que les spécialités turques sucuk et pastirma. Isla Délice, Çesnili, Sibel et d'autres marques. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Charcuterie de volaille et de bœuf pour pros | Fresco Marché</t>
+          <t>Charcuterie halal de volaille et bœuf | Fresco Marché</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -845,17 +845,17 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Délices de poulet et dinde, bacon de dinde, chorizo, saucisson, sucuk, pastirma… Charcuterie de volaille et de bœuf pour restaurants et snacks, commande pro.</t>
+          <t>Charcuterie halal : délices de poulet et dinde, bacon de dinde, chorizo, saucisson, sucuk, pastirma… Pour restaurants et snacks, en commande pro à Clichy.</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>Tout le rayon n'est pas halal : « halal » est retiré du titre et du texte. La description Google actuelle du site dit « Charcuterie halal » pour tout le rayon : à remplacer en priorité.</t>
+          <t>Tout le catalogue est halal (confirmé par Rachid le 13/10/2026). Citer l'organisme de certification sur le site renforcerait la confiance.</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="141" customHeight="1">
+    <row r="7" ht="100.5" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -879,7 +879,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Viandes pour la restauration rapide : viande de kebab de poulet Hünkar en 800 g (surgelé halal), lamelles de kebab bœuf-volaille Hünkar, steaks hachés 100 % pur bœuf et burgers de bœuf Biladi en 800 g, allumettes de poulet et dés de dinde halal, délices de volaille en tranches. Détail par espèce dans les rayons Volaille et Bœuf. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Viandes halal pour la restauration rapide : viande de kebab de poulet Hünkar en 800 g, lamelles de kebab bœuf-volaille Hünkar, steaks hachés 100 % pur bœuf et burgers de bœuf Biladi en 800 g, allumettes de poulet et dés de dinde, délices de volaille en tranches. Détail par espèce dans les rayons Volaille et Bœuf. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Kebab, burgers et steaks hachés pour pros | Fresco Marché</t>
+          <t>Viande halal : kebab, burgers, steaks hachés | Fresco Marché</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -899,17 +899,17 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Kebab de poulet Hünkar surgelé halal, lamelles bœuf-volaille, steaks hachés et burgers Biladi 800 g… Pour snacks et restaurants, commande pro à Clichy.</t>
+          <t>Viande halal pour snacks et restaurants : kebab de poulet Hünkar, lamelles bœuf-volaille, steaks hachés et burgers Biladi 800 g… Commande pro à Clichy.</t>
         </is>
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Aucune viande fraîche n'est en ligne dans ce rayon : si vous en vendez, publiez-la ; sinon, le nom « Boucherie » promet plus que ce qu'on trouve. « Halal » n'est écrit que pour les produits dont le nom le dit (kebab de poulet Hünkar, allumettes de poulet, dés de dinde). La description Google actuelle dit « surgelés halal » pour tout le rayon : elle est remplacée.</t>
+          <t>Aucune viande fraîche n'est en ligne dans ce rayon : si vous en vendez, publiez-la ; sinon, le nom « Boucherie » promet plus que ce qu'on trouve.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="87" customHeight="1">
+    <row r="8" ht="73.5" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -933,7 +933,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Volaille pour snacks et restaurants : viande de kebab de poulet Hünkar en 800 g (surgelé halal), allumettes de poulet et dés de dinde halal, délices et tranchés de poulet et de dinde pour les sandwichs. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Volaille halal pour snacks et restaurants : viande de kebab de poulet Hünkar en 800 g, allumettes de poulet et dés de dinde, délices et tranchés de poulet et de dinde pour les sandwichs. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Volaille pour snacks : kebab, poulet, dinde | Fresco Marché</t>
+          <t>Volaille halal : kebab, poulet, dinde | Fresco Marché</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Kebab de poulet Hünkar surgelé halal, allumettes de poulet, dés de dinde, délices de dinde et de poulet… La volaille des snacks et restaurants, commande pro.</t>
+          <t>Volaille halal : kebab de poulet Hünkar, allumettes de poulet, dés de dinde, délices de dinde et de poulet… Pour snacks et restaurants, commande pro à Clichy.</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>La marque s'écrit « Hunkar » sur les fiches kebab et « Hünkar » sur d'autres : choisir une seule orthographe. La description Google actuelle dit « Surgelés halal » pour tout le rayon : elle est remplacée.</t>
+          <t>La marque s'écrit « Hunkar » sur les fiches kebab et « Hünkar » sur d'autres : choisir une seule orthographe.</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr"/>
@@ -987,7 +987,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Bœuf pour burgers et kebabs : steaks hachés 100 % pur bœuf, burgers de bœuf nature ou à l'oignon Biladi en 800 g et lamelles de kebab bœuf et volaille Hünkar. Surgelés, prêts à cuisiner pour la restauration rapide. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Bœuf halal pour burgers et kebabs : steaks hachés 100 % pur bœuf, burgers de bœuf nature ou à l'oignon Biladi en 800 g et lamelles de kebab bœuf et volaille Hünkar. Surgelés, prêts à cuisiner pour la restauration rapide. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Steaks hachés et burgers de bœuf pour pros | Fresco Marché</t>
+          <t>Steaks hachés et burgers de bœuf halal | Fresco Marché</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1007,14 +1007,10 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Steaks hachés 100 % pur bœuf, burgers Biladi nature ou à l'oignon 800 g, lamelles de kebab Hünkar : le bœuf surgelé des snacks, en commande pro à Clichy.</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>La description Google actuelle dit « surgelés halal » ; aucun de ces produits ne l'indique dans son nom. Elle est remplacée.</t>
-        </is>
-      </c>
+          <t>Bœuf halal surgelé : steaks hachés 100 % pur bœuf, burgers Biladi nature ou à l'oignon 800 g, lamelles de kebab Hünkar. Pour snacks, commande pro à Clichy.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="87" customHeight="1">
@@ -1041,7 +1037,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Surgelés pour la restauration : frites en 1 kg et 2,5 kg, viande de kebab, steaks hachés et burgers de bœuf, légumes surgelés (haricots verts, chou-fleur, persil), crêpes feuilletées msemen et meloui, künefe et tartes Almondy pour les desserts. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Surgelés pour la restauration : frites en 1 kg et 2,5 kg, viandes halal (kebab, steaks hachés, burgers de bœuf), légumes surgelés (haricots verts, chou-fleur, persil), crêpes feuilletées msemen et meloui, künefe et tartes Almondy pour les desserts. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1299,7 +1295,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Produits turcs pour kebabs, durums et mezzés : concentré de tomate Tamek, galettes durum de 30 cm, viande de kebab de poulet Hünkar (surgelé halal), sucuk, pastirma de Kayseri, fromage traditionnel Erzurum et yaourt à la grecque en 1 kg. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Produits turcs pour kebabs, durums et mezzés : concentré de tomate Tamek, galettes durum de 30 cm, viande de kebab de poulet Hünkar, sucuk, pastirma de Kayseri, fromage traditionnel Erzurum et yaourt à la grecque en 1 kg. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1765,7 +1761,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Charcuterie turque pour sandwichs, pides et petits-déjeuners : sucuk en tranches, pastirma de Kayseri et pastirma sans çemen Isla Délice, salamis aux épices ou aux piments, salami volaille-bœuf au poivre Çesnili et saucisses bœuf-poulet Sibel. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
+          <t>Charcuterie turque halal pour sandwichs, pides et petits-déjeuners : sucuk en tranches, pastirma de Kayseri et pastirma sans çemen Isla Délice, salamis aux épices ou aux piments, salami volaille-bœuf au poivre Çesnili et saucisses bœuf-poulet Sibel. Commande en ligne réservée aux professionnels, livraison depuis notre dépôt de Clichy.</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1775,7 +1771,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Sucuk et pastirma : charcuterie turque pro | Fresco Marché</t>
+          <t>Sucuk et pastirma halal : charcuterie turque | Fresco Marché</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1785,14 +1781,10 @@
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Sucuk en tranches, pastirma de Kayseri, salamis aux épices, saucisses bœuf-poulet Sibel… La charcuterie turque des snacks et restaurants, en commande pro.</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>La description Google actuelle parle de « délices halal » : elle est remplacée, sans mention halal.</t>
-        </is>
-      </c>
+          <t>Sucuk en tranches, pastirma de Kayseri, salamis aux épices, saucisses bœuf-poulet Sibel… La charcuterie turque halal des snacks, en commande pro à Clichy.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="87" customHeight="1">
@@ -2062,7 +2054,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Tout le catalogue n'est pas halal : « halal » n'est jamais écrit pour un rayon entier, ni dans un titre Google. Il n'apparaît qu'à côté des produits dont le nom le dit (kebab de poulet Hünkar « surgelé halal », allumettes de poulet halal, dés de dinde halal).</t>
+          <t>Tout le catalogue est halal (confirmé par Rachid le 13/10/2026) : « halal » est mis en avant sur les rayons viande, volaille, bœuf, charcuterie et surgelés, là où les clients le cherchent. Il n'est pas ajouté là où il n'apporte rien (fruits, boissons, hygiène…).</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2135,53 +2127,53 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>« Halal » sur des rayons entiers (en ligne aujourd'hui)</t>
+          <t>Organisme de certification halal</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Les descriptions Google actuelles de Charcuterie (« Charcuterie halal en tranches »), Boucherie et Volaille (« surgelés halal »), Bœuf (« surgelés halal ») et Charcuterie turque (« délices halal ») présentent tout le rayon comme halal.</t>
+          <t>Aucune des 27 pages lues ni aucune description de produit ne nomme l'organisme de certification. 15 fiches disent « Certifié halal » sans le nommer.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Coller en priorité les nouvelles descriptions Google de ces 5 rayons (onglet Rayons, colonne J) : aucune ne présente le rayon entier comme halal.</t>
+          <t>Indiquer le ou les organismes de certification sur une page du site (par exemple « Nos engagements ») et dans les fiches : c'est ce que vérifient les restaurateurs, et cela renforce les recherches « halal certifié ».</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr"/>
     </row>
-    <row r="3" ht="87" customHeight="1">
+    <row r="3" ht="46.5" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>15 fiches « Certifié halal »</t>
+          <t>Prix visibles dans les filtres</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>15 fiches disent « Certifié halal » dans leur description sans que le nom du produit le précise : bacons de dinde, blanc de poulet doré, Deliss' Original, délices de dinde et de poulet, lardons de volaille, salami de dinde, Saveurdélice volaille et bœuf aux olives, Tosun pastirma, tranchettes piquantes, tranché de poulet et dinde.</t>
+          <t>Sur les pages rayon, le filtre « Precio » affiche le prix le plus élevé (7,50 € pour les fruits) et permet de filtrer par prix : les tarifs réservés aux pros sont visibles de tous.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Vérifier sur chaque emballage la mention et l'organisme de certification. Si ce n'est pas écrit sur l'emballage, retirer « Certifié halal » de la fiche.</t>
+          <t>Appli Search &amp; Discovery › Filtres : supprimer le filtre de prix.</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr"/>
     </row>
-    <row r="4" ht="46.5" customHeight="1">
+    <row r="4" ht="33" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Prix visibles dans les filtres</t>
+          <t>Filtres en espagnol</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Sur les pages rayon, le filtre « Precio » affiche le prix le plus élevé (7,50 € pour les fruits) et permet de filtrer par prix : les tarifs réservés aux pros sont visibles de tous.</t>
+          <t>Les filtres s'appellent « Disponibilidad » et « Precio ».</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Appli Search &amp; Discovery › Filtres : supprimer le filtre de prix.</t>
+          <t>Search &amp; Discovery › Filtres : renommer en « Disponibilité » (et « Prix » si le filtre est gardé).</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr"/>
@@ -2189,17 +2181,17 @@
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Filtres en espagnol</t>
+          <t>Poissonnerie</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Les filtres s'appellent « Disponibilidad » et « Precio ».</t>
+          <t>0 produit en ligne. La page est indexable et sa description Google promet « poissons et produits de la mer frais et surgelés ».</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Search &amp; Discovery › Filtres : renommer en « Disponibilité » (et « Prix » si le filtre est gardé).</t>
+          <t>Masquer la collection du canal Boutique en ligne tant qu'elle est vide, ou publier les produits.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
@@ -2207,17 +2199,17 @@
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Poissonnerie</t>
+          <t>Arrivages Rungis</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0 produit en ligne. La page est indexable et sa description Google promet « poissons et produits de la mer frais et surgelés ».</t>
+          <t>0 produit en ligne. Le texte annonce « produits arrivés ce matin directement de Rungis… mise à jour chaque matin à 00h01 ».</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Masquer la collection du canal Boutique en ligne tant qu'elle est vide, ou publier les produits.</t>
+          <t>Même chose que Poissonnerie. Une fois alimenté, ce rayon vaut la peine d'être travaillé : « Rungis » est un argument fort.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
@@ -2225,92 +2217,74 @@
     <row r="7" ht="33" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Arrivages Rungis</t>
+          <t>Asie</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>0 produit en ligne. Le texte annonce « produits arrivés ce matin directement de Rungis… mise à jour chaque matin à 00h01 ».</t>
+          <t>2 produits en ligne (aloe vera, coco à boire). La description Google promet « sauces, condiments et ingrédients » d'Asie.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Même chose que Poissonnerie. Une fois alimenté, ce rayon vaut la peine d'être travaillé : « Rungis » est un argument fort.</t>
+          <t>Publier les produits asiatiques, ou masquer le rayon en attendant.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="33" customHeight="1">
+    <row r="8" ht="46.5" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Asie</t>
+          <t>Note interne sur les autres rayons</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2 produits en ligne (aloe vera, coco à boire). La description Google promet « sauces, condiments et ingrédients » d'Asie.</t>
+          <t>52 autres rayons, hors de ce tableau, affichent encore « Collection automatique … Parent : … » (ex. Agrumes, Bacon-lardons, Bouillons, Cafés-thés).</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Publier les produits asiatiques, ou masquer le rayon en attendant.</t>
+          <t>Après ces 25 rayons : écrire un texte court pour les sous-rayons utiles, et vider la description des autres.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
     </row>
-    <row r="9" ht="46.5" customHeight="1">
+    <row r="9" ht="33" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Note interne sur les autres rayons</t>
+          <t>Produits non publiés</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>52 autres rayons, hors de ce tableau, affichent encore « Collection automatique … Parent : … » (ex. Agrumes, Bacon-lardons, Bouillons, Cafés-thés).</t>
+          <t>Beaucoup de produits des rayons ne sont pas publiés en ligne (ex. Boissons : 13 en ligne sur 182 dans l'admin).</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Après ces 25 rayons : écrire un texte court pour les sous-rayons utiles, et vider la description des autres.</t>
+          <t>Publier les produits prêts : chaque rayon en devient plus utile pour les clients et pour Google.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
     </row>
-    <row r="10" ht="33" customHeight="1">
+    <row r="10" ht="46.5" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Produits non publiés</t>
+          <t>Nom de produit à corriger</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Beaucoup de produits des rayons ne sont pas publiés en ligne (ex. Boissons : 13 en ligne sur 182 dans l'admin).</t>
+          <t>« Cerneaux de noix extra invalide 250g Profruit » (le mot « invalide » vient sans doute de l'import) ; « COUCOUS MOYEN DARI 1KG » (faute et majuscules).</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Publier les produits prêts : chaque rayon en devient plus utile pour les clients et pour Google.</t>
+          <t>Renommer : « Cerneaux de noix extra 250 g Profruit », « Couscous moyen Dari 1 kg ».</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="46.5" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Nom de produit à corriger</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>« Cerneaux de noix extra invalide 250g Profruit » (le mot « invalide » vient sans doute de l'import) ; « COUCOUS MOYEN DARI 1KG » (faute et majuscules).</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Renommer : « Cerneaux de noix extra 250 g Profruit », « Couscous moyen Dari 1 kg ».</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>